<commit_message>
fix: update 698 stale standard references across all document types
Online-verified accuracy updates (2026-02-08):
- PCI DSS v4.0 → v4.0.1 (sole version since Jan 2025)
- CIS Controls v8 → v8.1 (released June 2024)
- OWASP Top 10 2021 → 2025 (finalized Jan 2026)
- NIST SP 800-88 → Rev. 2 (finalized Sep 2025, Rev. 1 withdrawn)
- NIST CSF → 2.0 (released Feb 2024)
- Azure AD → Microsoft Entra ID (formerly Azure AD)

Scope: 254 IMP-UG + 68 GOV-POL + 70 Python generators + regenerated workbooks

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/isms-core-framework/A.5-organizational-controls/isms-a.5.14-information-transfer/WKBK/90_workbooks/ISMS-IMP-A.5.14.1_Transfer_Rules_and_Procedures_20260208.xlsx
+++ b/isms-core-framework/A.5-organizational-controls/isms-a.5.14-information-transfer/WKBK/90_workbooks/ISMS-IMP-A.5.14.1_Transfer_Rules_and_Procedures_20260208.xlsx
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Azure AD SSO</t>
+          <t>Microsoft Entra ID (formerly Azure AD) SSO</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Azure AD + MFA</t>
+          <t>Microsoft Entra ID (formerly Azure AD) + MFA</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Azure AD + MFA</t>
+          <t>Microsoft Entra ID (formerly Azure AD) + MFA</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Azure AD + MFA</t>
+          <t>Microsoft Entra ID (formerly Azure AD) + MFA</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Azure AD authentication</t>
+          <t>Microsoft Entra ID (formerly Azure AD) authentication</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">

</xml_diff>